<commit_message>
Exclude Coupang ad spend from team ROAS
Coupang ads are run by the team lead, who is also out of scope for the
team-member KPI. Chae's ROAS stays 0 as in the source sheet; Shin's ROAS
excludes WING(Miyu) ad spend.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U57HqgEQfdTuX1dvSuHD8X
</commit_message>
<xml_diff>
--- a/kpi/2026-09/2026-09_팀원_KPI.xlsx
+++ b/kpi/2026-09/2026-09_팀원_KPI.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,7 +127,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -587,8 +586,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>종합점수
-(보정)</t>
+          <t>종합점수</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -630,10 +628,10 @@
         <v>-0.2920361320777328</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>6530577</v>
+        <v>0</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>4.387298090199381</v>
+        <v>0</v>
       </c>
       <c r="I5" s="9" t="n">
         <v>0</v>
@@ -642,7 +640,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="10" t="n">
-        <v>0.3627931136363637</v>
+        <v>0.1627931136363636</v>
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
@@ -680,10 +678,10 @@
         <v>-0.07430061740556182</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>4387455</v>
+        <v>2438281</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>6.044434415851558</v>
+        <v>10.87638545352238</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>3</v>
@@ -780,28 +778,25 @@
         <v>-0.2685607024107091</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>11677378</v>
-      </c>
-      <c r="H8" s="15" t="n">
-        <v>5.301523595450965</v>
+        <v>3197627</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>※ 종합점수(보정): 채동훈 광고비가 시트에서 '김혜원' 행(WING(신우)·로켓배송(직매입))에 입력돼 ROAS가 0으로 계산됨 → 담당자 기준으로 바로잡아 재계산</t>
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>※ 쿠팡 광고비는 김혜원 부장 운영 → 팀원 ROAS에서 제외 (신희섭 WING(미유) 광고비 195만원 제외, 점수 영향 없음)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>※ 광고비는 KPI 시트 기준(VAT 포함 추정). 월간성과보고의 광고비와 약 10% 차이</t>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>※ 김혜원 부장은 팀원 KPI 평가 대상에서 제외 / 광고비는 KPI 시트 기준(VAT 포함 추정)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>※ 3명 모두 매출 달성률 50% 미만으로 등급 D (하한선 규정). 9월 핫팩 목표(시즌 목표)가 실제 핫팩 출고 시점보다 앞서 잡힌 영향이 큼</t>
         </is>
@@ -818,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -874,7 +869,7 @@
           <t>담당채널 매출</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B4" s="17" t="n">
         <v>0.5</v>
       </c>
       <c r="C4" s="5" t="n">
@@ -896,20 +891,20 @@
           <t>광고 ROAS</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="20" t="n">
-        <v>4.387298090199381</v>
+      <c r="D5" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1.462432696733127</v>
+        <v>0</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -918,13 +913,13 @@
           <t>딜 참여</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="7" t="n">
@@ -940,13 +935,13 @@
           <t>SNS·부서 협업</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="7" t="n">
@@ -970,8 +965,8 @@
           <t>등급 D</t>
         </is>
       </c>
-      <c r="F8" s="21" t="n">
-        <v>0.3627931136363637</v>
+      <c r="F8" s="20" t="n">
+        <v>0.1627931136363636</v>
       </c>
     </row>
     <row r="10">
@@ -1022,11 +1017,9 @@
         <v>0.9097914814814815</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>4181846</v>
-      </c>
-      <c r="F11" s="8" t="n">
-        <v>5.874049403062666</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1372,114 +1365,94 @@
       </c>
       <c r="F29" s="4" t="n"/>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>로켓배송(직매입)</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="5" t="n">
-        <v>2348731</v>
-      </c>
-      <c r="F30" s="8" t="n">
-        <v>0</v>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>9월 딜</t>
+        </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="inlineStr">
-        <is>
-          <t>9월 딜</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>등록된 딜 없음</t>
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>9월 성과·이슈</t>
+        </is>
+      </c>
+    </row>
     <row r="35">
-      <c r="A35" s="22" t="inlineStr">
-        <is>
-          <t>9월 성과·이슈</t>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>▶ 쿠팡 WING(신우) 2,456만원 — 목표 2,700만원 대비 91%, 담당 매출의 86%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>▶ 쿠팡 WING(신우) 2,456만원 — 목표 2,700만원 대비 91%, 담당 매출의 86%</t>
+          <t>▶ 쿠팡 로켓배송(직매입)-핫팩 목표 2,800만원 대비 실적 0원 → 9월 미달의 최대 원인 (발주 일정 확인)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>▶ 쿠팡 로켓배송(직매입)-핫팩 목표 2,800만원 대비 실적 0원 → 9월 미달의 최대 원인 (발주 일정 확인)</t>
+          <t>▶ 카카오 선물하기·쇼핑하기·메이커스 핫팩 목표 1,500만원 대비 62만원</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>▶ 카카오 선물하기·쇼핑하기·메이커스 핫팩 목표 1,500만원 대비 62만원</t>
+          <t>▶ 딜 0건 (목표 월 3회), SNS 협업 0건 → 매출 외 항목 점수 0점</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>▶ 딜 0건 (목표 월 3회), SNS 협업 0건 → 매출 외 항목 점수 0점</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>▶ 손익: 쿠팡 직매입(미유) 광고비 214만원 / 매출 12만원 → 영업손실 -208만원</t>
+          <t>▶ 운영 광고 없음(쿠팡 광고는 김혜원 부장 운영) → ROAS 항목(20%) 0점, 최고 점수 0.8로 구조적 불리</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>10월 실행 과제</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="inlineStr">
-        <is>
-          <t>10월 실행 과제</t>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>□ 로켓배송(직매입)-핫팩 10월 발주 확정 (목표 2,800만원)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>□ 로켓배송(직매입)-핫팩 10월 발주 확정 (목표 2,800만원)</t>
+          <t>□ 카카오 핫팩 3개 채널 시즌 기획전 1건 이상</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>□ 카카오 핫팩 3개 채널 시즌 기획전 1건 이상</t>
+          <t>□ 딜 월 3회 등록 (쿠팡·카카오·오늘의집)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>□ 딜 월 3회 등록 (쿠팡·카카오·오늘의집)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>□ 쿠팡 직매입(미유) 광고 중단 또는 축소</t>
+          <t>□ 카카오·오늘의집 자체 프로모션 기획 1건</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1523,7 @@
           <t>담당채널 매출</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B4" s="17" t="n">
         <v>0.5</v>
       </c>
       <c r="C4" s="5" t="n">
@@ -1572,17 +1545,17 @@
           <t>광고 ROAS</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="20" t="n">
-        <v>6.044434415851558</v>
+      <c r="D5" s="19" t="n">
+        <v>10.87638545352238</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>2.014811471950519</v>
+        <v>3.625461817840793</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>0.2</v>
@@ -1594,13 +1567,13 @@
           <t>딜 참여</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="7" t="n">
@@ -1616,13 +1589,13 @@
           <t>SNS·부서 협업</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="7" t="n">
@@ -1646,7 +1619,7 @@
           <t>등급 D</t>
         </is>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="F8" s="20" t="n">
         <v>0.4402951447054818</v>
       </c>
     </row>
@@ -1714,15 +1687,13 @@
       <c r="C12" s="5" t="n">
         <v>13310740</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="22" t="n">
         <v>1.331074</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>1900777</v>
-      </c>
-      <c r="F12" s="8" t="n">
-        <v>7.002788859503245</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1824,11 +1795,9 @@
         <v>0.1750533333333333</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>48397</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>10.85108581110399</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1913,7 +1882,7 @@
       <c r="F21" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>9월 딜</t>
         </is>
@@ -1941,7 +1910,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>9월 성과·이슈</t>
         </is>
@@ -1971,7 +1940,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>▶ 딜 3건 달성(목표 충족), ROAS 6.04로 우수, SNS 협업 0건</t>
+          <t>▶ 딜 3건 달성(목표 충족), ROAS 10.88(쿠팡 광고 제외)로 우수, SNS 협업 0건</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1952,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>10월 실행 과제</t>
         </is>
@@ -2077,7 +2046,7 @@
           <t>담당채널 매출</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B4" s="17" t="n">
         <v>0.5</v>
       </c>
       <c r="C4" s="5" t="n">
@@ -2099,13 +2068,13 @@
           <t>광고 ROAS</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="19" t="n">
         <v>8.871611887071243</v>
       </c>
       <c r="E5" s="7" t="n">
@@ -2121,13 +2090,13 @@
           <t>딜 참여</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="7" t="n">
@@ -2143,13 +2112,13 @@
           <t>SNS·부서 협업</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="7" t="n">
@@ -2173,7 +2142,7 @@
           <t>등급 D</t>
         </is>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="F8" s="20" t="n">
         <v>0.4724410070422535</v>
       </c>
     </row>
@@ -2360,7 +2329,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>SSG-핫팩</t>
+          <t>옥션-핫팩</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
@@ -2380,7 +2349,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>옥션-핫팩</t>
+          <t>SSG-핫팩</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
@@ -2409,7 +2378,7 @@
       <c r="C20" s="5" t="n">
         <v>1892113</v>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="22" t="n">
         <v>1.892113</v>
       </c>
       <c r="E20" s="5" t="n">
@@ -2476,7 +2445,7 @@
       <c r="F23" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>9월 딜</t>
         </is>
@@ -2504,7 +2473,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>9월 성과·이슈</t>
         </is>
@@ -2546,7 +2515,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="inlineStr">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>10월 실행 과제</t>
         </is>

</xml_diff>

<commit_message>
Keep WING(Miyu) ad spend with Shin per ad sheet ownership
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U57HqgEQfdTuX1dvSuHD8X
</commit_message>
<xml_diff>
--- a/kpi/2026-09/2026-09_팀원_KPI.xlsx
+++ b/kpi/2026-09/2026-09_팀원_KPI.xlsx
@@ -678,10 +678,10 @@
         <v>-0.07430061740556182</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2438281</v>
+        <v>4387455</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>10.87638545352238</v>
+        <v>6.044434415851558</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>3</v>
@@ -778,13 +778,13 @@
         <v>-0.2685607024107091</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>3197627</v>
+        <v>5146801</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>※ 쿠팡 광고비는 김혜원 부장 운영 → 팀원 ROAS에서 제외 (신희섭 WING(미유) 광고비 195만원 제외, 점수 영향 없음)</t>
+          <t>※ 광고비는 「월별광고비」 담당자 기준 (쿠팡 WING(신우)·로켓배송 광고는 김혜원 부장, WING(미유)는 신희섭)</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>▶ 운영 광고 없음(쿠팡 광고는 김혜원 부장 운영) → ROAS 항목(20%) 0점, 최고 점수 0.8로 구조적 불리</t>
+          <t>▶ 운영 광고 없음(쿠팡 WING(신우)·로켓배송 광고는 김혜원 부장 운영) → ROAS 항목(20%) 0점, 최고 점수 0.8로 구조적 불리</t>
         </is>
       </c>
     </row>
@@ -1552,10 +1552,10 @@
         <v>3</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>10.87638545352238</v>
+        <v>6.044434415851558</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>3.625461817840793</v>
+        <v>2.014811471950519</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>0.2</v>
@@ -1691,9 +1691,11 @@
         <v>1.331074</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="4" t="n"/>
+        <v>1900777</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>7.002788859503245</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1795,9 +1797,11 @@
         <v>0.1750533333333333</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="4" t="n"/>
+        <v>48397</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>10.85108581110399</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1940,7 +1944,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>▶ 딜 3건 달성(목표 충족), ROAS 10.88(쿠팡 광고 제외)로 우수, SNS 협업 0건</t>
+          <t>▶ 딜 3건 달성(목표 충족), ROAS 6.04로 우수, SNS 협업 0건</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2333,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>옥션-핫팩</t>
+          <t>SSG-핫팩</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
@@ -2349,7 +2353,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>SSG-핫팩</t>
+          <t>옥션-핫팩</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">

</xml_diff>